<commit_message>
Evaluate logistic model using area between curves
</commit_message>
<xml_diff>
--- a/LogisticModel.xlsx
+++ b/LogisticModel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6957AED7-077E-104F-BF94-BDF56BF2AFA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{418D80A2-755D-1D49-9F73-65868174868A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="-23500" windowWidth="38400" windowHeight="22400" activeTab="1" xr2:uid="{EA72EE1C-EB9E-194F-A03F-497BA5E072C1}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14480" activeTab="2" xr2:uid="{EA72EE1C-EB9E-194F-A03F-497BA5E072C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Biofermentation semaine 3 ex" sheetId="1" r:id="rId1"/>
@@ -20,11 +20,7 @@
     <sheet name="8F3_exer_w3" sheetId="6" r:id="rId5"/>
     <sheet name="8F3_labo5_o2" sheetId="7" r:id="rId6"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId7"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -45,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="21">
   <si>
     <t>Temps (h)</t>
   </si>
@@ -148,6 +144,9 @@
   <si>
     <t>Interpolée 2B</t>
   </si>
+  <si>
+    <t>A-b-k</t>
+  </si>
 </sst>
 </file>
 
@@ -199,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -217,15 +216,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -400,7 +409,7 @@
             <c:numRef>
               <c:f>'Biofermentation semaine 3 ex'!$B$6:$B$13</c:f>
               <c:numCache>
-                <c:formatCode>0\.0</c:formatCode>
+                <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0" formatCode="General">
                   <c:v>1.5</c:v>
@@ -429,7 +438,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="1"/>
+          <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-04CF-C14A-8E79-0D5BDBE92856}"/>
@@ -1240,7 +1249,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="10"/>
-          <c:min val="0"/>
+          <c:min val="1"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -2544,10 +2553,10 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.8367300212958384"/>
+          <c:x val="0.75469784719754351"/>
           <c:y val="0.11532956042961007"/>
-          <c:w val="0.13335407206351171"/>
-          <c:h val="0.22564108358287194"/>
+          <c:w val="0.21538624616180663"/>
+          <c:h val="0.23170416734365798"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -6063,7 +6072,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8671034" cy="6284310"/>
+    <xdr:ext cx="8669461" cy="6281557"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Graphique 1">
@@ -6209,272 +6218,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="8F3_exer_w3"/>
-      <sheetName val="8F3_labo5_o2"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="6">
-          <cell r="B6" t="str">
-            <v>y</v>
-          </cell>
-          <cell r="C6" t="str">
-            <v>y^</v>
-          </cell>
-          <cell r="D6" t="str">
-            <v>y^'</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7">
-            <v>0</v>
-          </cell>
-          <cell r="B7">
-            <v>1.5</v>
-          </cell>
-          <cell r="C7">
-            <v>1.5123225937450893</v>
-          </cell>
-          <cell r="D7">
-            <v>1.4999999999999922</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8">
-            <v>5</v>
-          </cell>
-          <cell r="B8">
-            <v>2</v>
-          </cell>
-          <cell r="C8">
-            <v>1.6724969976216613</v>
-          </cell>
-          <cell r="D8">
-            <v>1.6604472071404059</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9">
-            <v>9</v>
-          </cell>
-          <cell r="B9">
-            <v>3.5</v>
-          </cell>
-          <cell r="C9">
-            <v>2.7560682823620697</v>
-          </cell>
-          <cell r="D9">
-            <v>2.7458639913859049</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10">
-            <v>13</v>
-          </cell>
-          <cell r="B10">
-            <v>6.2</v>
-          </cell>
-          <cell r="C10">
-            <v>6.5053452039466082</v>
-          </cell>
-          <cell r="D10">
-            <v>6.5015265461084493</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11">
-            <v>16</v>
-          </cell>
-          <cell r="B11">
-            <v>8.1999999999999993</v>
-          </cell>
-          <cell r="C11">
-            <v>8.8838196032012675</v>
-          </cell>
-          <cell r="D11">
-            <v>8.8840518771186012</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12">
-            <v>20</v>
-          </cell>
-          <cell r="B12">
-            <v>9.4</v>
-          </cell>
-          <cell r="C12">
-            <v>9.7643757571501517</v>
-          </cell>
-          <cell r="D12">
-            <v>9.7661077625288115</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13">
-            <v>24</v>
-          </cell>
-          <cell r="B13">
-            <v>9.8000000000000007</v>
-          </cell>
-          <cell r="C13">
-            <v>9.8835942888271155</v>
-          </cell>
-          <cell r="D13">
-            <v>9.8855293429062225</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14">
-            <v>28</v>
-          </cell>
-          <cell r="B14">
-            <v>9.9</v>
-          </cell>
-          <cell r="C14">
-            <v>9.8980403419246183</v>
-          </cell>
-          <cell r="D14">
-            <v>9.8999999999999897</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1">
-        <row r="6">
-          <cell r="B6" t="str">
-            <v>y</v>
-          </cell>
-          <cell r="C6" t="str">
-            <v>y^</v>
-          </cell>
-          <cell r="D6" t="str">
-            <v>y^'</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7">
-            <v>0</v>
-          </cell>
-          <cell r="B7">
-            <v>105.1</v>
-          </cell>
-          <cell r="C7">
-            <v>103.73943847719816</v>
-          </cell>
-          <cell r="D7">
-            <v>104.78728956603497</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8">
-            <v>0.5</v>
-          </cell>
-          <cell r="B8">
-            <v>103.7</v>
-          </cell>
-          <cell r="C8">
-            <v>101.01058733442666</v>
-          </cell>
-          <cell r="D8">
-            <v>101.94282214909731</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9">
-            <v>1</v>
-          </cell>
-          <cell r="B9">
-            <v>98.4</v>
-          </cell>
-          <cell r="C9">
-            <v>93.426218607705962</v>
-          </cell>
-          <cell r="D9">
-            <v>94.037118029492092</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10">
-            <v>1.5</v>
-          </cell>
-          <cell r="B10">
-            <v>85.5</v>
-          </cell>
-          <cell r="C10">
-            <v>75.859614230350189</v>
-          </cell>
-          <cell r="D10">
-            <v>75.726249769058299</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11">
-            <v>2</v>
-          </cell>
-          <cell r="B11">
-            <v>51.6</v>
-          </cell>
-          <cell r="C11">
-            <v>48.052102529360404</v>
-          </cell>
-          <cell r="D11">
-            <v>46.740586264069663</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12">
-            <v>2.5</v>
-          </cell>
-          <cell r="B12">
-            <v>1</v>
-          </cell>
-          <cell r="C12">
-            <v>22.654543434140322</v>
-          </cell>
-          <cell r="D12">
-            <v>20.266980509696833</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13">
-            <v>3</v>
-          </cell>
-          <cell r="B13">
-            <v>0.8</v>
-          </cell>
-          <cell r="C13">
-            <v>8.7614609499045759</v>
-          </cell>
-          <cell r="D13">
-            <v>5.7852743338517207</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14">
-            <v>3.5</v>
-          </cell>
-          <cell r="B14">
-            <v>0.3</v>
-          </cell>
-          <cell r="C14">
-            <v>3.199141176011191</v>
-          </cell>
-          <cell r="D14">
-            <v>-1.271043396478877E-2</v>
-          </cell>
-        </row>
-      </sheetData>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6794,7 +6537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AFA3DA8-A952-DB4B-A693-8E3526DC5924}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -6802,9 +6545,11 @@
     <col min="3" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.83203125" customWidth="1"/>
     <col min="7" max="8" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="12" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
@@ -6814,8 +6559,14 @@
       <c r="E1">
         <v>1.5</v>
       </c>
+      <c r="L1">
+        <v>1.5</v>
+      </c>
+      <c r="M1">
+        <v>1.5</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
@@ -6825,18 +6576,43 @@
       <c r="E2">
         <v>8.4</v>
       </c>
+      <c r="L2">
+        <v>8.4</v>
+      </c>
+      <c r="M2">
+        <v>8.4</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="L3">
+        <v>12.269617706237399</v>
+      </c>
+      <c r="M3">
+        <v>12.3246333771056</v>
+      </c>
+      <c r="N3" t="s">
+        <v>20</v>
+      </c>
+      <c r="O3">
+        <f>M2-K6-M1</f>
+        <v>5.4</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="L4">
+        <v>1.8809533698123699</v>
+      </c>
+      <c r="M4">
+        <v>2.68210649695129</v>
+      </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
@@ -6861,8 +6637,20 @@
       <c r="H5" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="J5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>0</v>
       </c>
@@ -6887,8 +6675,23 @@
       <c r="H6" s="2">
         <v>1.5</v>
       </c>
+      <c r="J6" s="2">
+        <v>0</v>
+      </c>
+      <c r="K6" s="10">
+        <f>B6</f>
+        <v>1.5</v>
+      </c>
+      <c r="L6" s="10">
+        <f>L$1+L$2*(1/(1+EXP(($J6-L$3)/(-1*L$4))))</f>
+        <v>1.5123225937450893</v>
+      </c>
+      <c r="M6" s="10">
+        <f>M$1+M$2*(1/(1+EXP(($J6-M$3)/(-1*M$4))))</f>
+        <v>1.5839989900710201</v>
+      </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -6913,8 +6716,23 @@
       <c r="H7" s="2">
         <v>1.79</v>
       </c>
+      <c r="J7" s="2">
+        <v>0.13218298714353499</v>
+      </c>
+      <c r="K7" s="10">
+        <f>1.5+0.1*J7</f>
+        <v>1.5132182987143534</v>
+      </c>
+      <c r="L7" s="10">
+        <f t="shared" ref="L7:M22" si="0">L$1+L$2*(1/(1+EXP(($J7-L$3)/(-1*L$4))))</f>
+        <v>1.5132182987143532</v>
+      </c>
+      <c r="M7" s="10">
+        <f t="shared" si="0"/>
+        <v>1.5881978868121776</v>
+      </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>9</v>
       </c>
@@ -6939,8 +6757,23 @@
       <c r="H8" s="2">
         <v>3.07</v>
       </c>
+      <c r="J8" s="2">
+        <v>5</v>
+      </c>
+      <c r="K8" s="11">
+        <f>B7</f>
+        <v>2</v>
+      </c>
+      <c r="L8" s="10">
+        <f t="shared" si="0"/>
+        <v>1.6724969976216613</v>
+      </c>
+      <c r="M8" s="10">
+        <f t="shared" si="0"/>
+        <v>2.0138530442580507</v>
+      </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>13</v>
       </c>
@@ -6965,8 +6798,19 @@
       <c r="H9" s="2">
         <v>6.33</v>
       </c>
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
+      <c r="K9" s="12">
+        <f>1.5+0.1*J9</f>
+        <v>1.5</v>
+      </c>
+      <c r="M9" s="10">
+        <f t="shared" si="0"/>
+        <v>1.5839989900710201</v>
+      </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>16</v>
       </c>
@@ -6991,8 +6835,19 @@
       <c r="H10" s="2">
         <v>8.52</v>
       </c>
+      <c r="J10" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="K10" s="12">
+        <f t="shared" ref="K10:K34" si="1">1.5+0.1*J10</f>
+        <v>1.52</v>
+      </c>
+      <c r="M10" s="10">
+        <f t="shared" si="0"/>
+        <v>1.5904320871158724</v>
+      </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>20</v>
       </c>
@@ -7017,8 +6872,19 @@
       <c r="H11" s="2">
         <v>9.6300000000000008</v>
       </c>
+      <c r="J11" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="K11" s="12">
+        <f t="shared" si="1"/>
+        <v>1.54</v>
+      </c>
+      <c r="M11" s="10">
+        <f t="shared" si="0"/>
+        <v>1.5973520979079312</v>
+      </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>24</v>
       </c>
@@ -7043,8 +6909,19 @@
       <c r="H12" s="2">
         <v>9.86</v>
       </c>
+      <c r="J12" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="K12" s="12">
+        <f t="shared" si="1"/>
+        <v>1.56</v>
+      </c>
+      <c r="M12" s="10">
+        <f t="shared" si="0"/>
+        <v>1.6047949611111947</v>
+      </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>28</v>
       </c>
@@ -7068,6 +6945,290 @@
       </c>
       <c r="H13" s="2">
         <v>9.9</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="K13" s="12">
+        <f t="shared" si="1"/>
+        <v>1.58</v>
+      </c>
+      <c r="M13" s="10">
+        <f t="shared" si="0"/>
+        <v>1.6127991229945868</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="J14" s="2">
+        <v>1</v>
+      </c>
+      <c r="K14" s="12">
+        <f t="shared" si="1"/>
+        <v>1.6</v>
+      </c>
+      <c r="M14" s="10">
+        <f t="shared" si="0"/>
+        <v>1.6214056893310302</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="J15" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="K15" s="12">
+        <f t="shared" si="1"/>
+        <v>1.62</v>
+      </c>
+      <c r="M15" s="10">
+        <f t="shared" si="0"/>
+        <v>1.6306585827354179</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="J16" s="2">
+        <v>1.4</v>
+      </c>
+      <c r="K16" s="12">
+        <f t="shared" si="1"/>
+        <v>1.64</v>
+      </c>
+      <c r="M16" s="10">
+        <f t="shared" si="0"/>
+        <v>1.6406047049588284</v>
+      </c>
+    </row>
+    <row r="17" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J17" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="K17" s="12">
+        <f t="shared" si="1"/>
+        <v>1.6600000000000001</v>
+      </c>
+      <c r="M17" s="10">
+        <f t="shared" si="0"/>
+        <v>1.6512941035000683</v>
+      </c>
+    </row>
+    <row r="18" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J18" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="K18" s="12">
+        <f t="shared" si="1"/>
+        <v>1.68</v>
+      </c>
+      <c r="M18" s="10">
+        <f t="shared" si="0"/>
+        <v>1.6627801417142061</v>
+      </c>
+    </row>
+    <row r="19" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J19" s="2">
+        <v>2</v>
+      </c>
+      <c r="K19" s="12">
+        <f t="shared" si="1"/>
+        <v>1.7</v>
+      </c>
+      <c r="M19" s="10">
+        <f t="shared" si="0"/>
+        <v>1.6751196713883938</v>
+      </c>
+    </row>
+    <row r="20" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J20" s="2">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="K20" s="12">
+        <f t="shared" si="1"/>
+        <v>1.72</v>
+      </c>
+      <c r="M20" s="10">
+        <f t="shared" si="0"/>
+        <v>1.6883732065151926</v>
+      </c>
+    </row>
+    <row r="21" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J21" s="2">
+        <v>2.4</v>
+      </c>
+      <c r="K21" s="12">
+        <f t="shared" si="1"/>
+        <v>1.74</v>
+      </c>
+      <c r="M21" s="10">
+        <f t="shared" si="0"/>
+        <v>1.7026050967199733</v>
+      </c>
+    </row>
+    <row r="22" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J22" s="2">
+        <v>2.6</v>
+      </c>
+      <c r="K22" s="12">
+        <f t="shared" si="1"/>
+        <v>1.76</v>
+      </c>
+      <c r="M22" s="10">
+        <f t="shared" si="0"/>
+        <v>1.7178836984890391</v>
+      </c>
+    </row>
+    <row r="23" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J23" s="2">
+        <v>2.8</v>
+      </c>
+      <c r="K23" s="12">
+        <f t="shared" si="1"/>
+        <v>1.78</v>
+      </c>
+      <c r="M23" s="10">
+        <f t="shared" ref="M23:M34" si="2">M$1+M$2*(1/(1+EXP(($J23-M$3)/(-1*M$4))))</f>
+        <v>1.7342815419963737</v>
+      </c>
+    </row>
+    <row r="24" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J24" s="2">
+        <v>3</v>
+      </c>
+      <c r="K24" s="12">
+        <f t="shared" si="1"/>
+        <v>1.8</v>
+      </c>
+      <c r="M24" s="10">
+        <f t="shared" si="2"/>
+        <v>1.7518754909371519</v>
+      </c>
+    </row>
+    <row r="25" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J25" s="2">
+        <v>3.2</v>
+      </c>
+      <c r="K25" s="12">
+        <f t="shared" si="1"/>
+        <v>1.82</v>
+      </c>
+      <c r="M25" s="10">
+        <f t="shared" si="2"/>
+        <v>1.7707468923437055</v>
+      </c>
+    </row>
+    <row r="26" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J26" s="2">
+        <v>3.4</v>
+      </c>
+      <c r="K26" s="12">
+        <f t="shared" si="1"/>
+        <v>1.84</v>
+      </c>
+      <c r="M26" s="10">
+        <f t="shared" si="2"/>
+        <v>1.7909817128836134</v>
+      </c>
+    </row>
+    <row r="27" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J27" s="2">
+        <v>3.6</v>
+      </c>
+      <c r="K27" s="12">
+        <f t="shared" si="1"/>
+        <v>1.86</v>
+      </c>
+      <c r="M27" s="10">
+        <f t="shared" si="2"/>
+        <v>1.8126706576201035</v>
+      </c>
+    </row>
+    <row r="28" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J28" s="2">
+        <v>3.8</v>
+      </c>
+      <c r="K28" s="12">
+        <f t="shared" si="1"/>
+        <v>1.88</v>
+      </c>
+      <c r="M28" s="10">
+        <f t="shared" si="2"/>
+        <v>1.8359092666535222</v>
+      </c>
+    </row>
+    <row r="29" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J29" s="2">
+        <v>4</v>
+      </c>
+      <c r="K29" s="12">
+        <f t="shared" si="1"/>
+        <v>1.9</v>
+      </c>
+      <c r="M29" s="10">
+        <f t="shared" si="2"/>
+        <v>1.860797984462522</v>
+      </c>
+    </row>
+    <row r="30" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J30" s="2">
+        <v>4.2</v>
+      </c>
+      <c r="K30" s="12">
+        <f t="shared" si="1"/>
+        <v>1.92</v>
+      </c>
+      <c r="M30" s="10">
+        <f t="shared" si="2"/>
+        <v>1.8874421961302827</v>
+      </c>
+    </row>
+    <row r="31" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J31" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="K31" s="12">
+        <f t="shared" si="1"/>
+        <v>1.94</v>
+      </c>
+      <c r="M31" s="10">
+        <f t="shared" si="2"/>
+        <v>1.9159522239827265</v>
+      </c>
+    </row>
+    <row r="32" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J32" s="2">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="K32" s="12">
+        <f t="shared" si="1"/>
+        <v>1.96</v>
+      </c>
+      <c r="M32" s="10">
+        <f t="shared" si="2"/>
+        <v>1.9464432774937559</v>
+      </c>
+    </row>
+    <row r="33" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J33" s="2">
+        <v>4.8</v>
+      </c>
+      <c r="K33" s="12">
+        <f t="shared" si="1"/>
+        <v>1.98</v>
+      </c>
+      <c r="M33" s="10">
+        <f t="shared" si="2"/>
+        <v>1.9790353486423826</v>
+      </c>
+    </row>
+    <row r="34" spans="10:13" x14ac:dyDescent="0.2">
+      <c r="J34" s="2">
+        <v>5</v>
+      </c>
+      <c r="K34" s="12">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="M34" s="10">
+        <f t="shared" si="2"/>
+        <v>2.0138530442580507</v>
       </c>
     </row>
   </sheetData>
@@ -7077,9 +7238,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBA9180D-0927-4B40-8D2B-EAD906206BCB}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.83203125" bestFit="1" customWidth="1"/>
@@ -7193,7 +7355,7 @@
         <v>105.1</v>
       </c>
       <c r="G6" s="4">
-        <f>G$1+G$2*(1/(1+EXP(($A6-G$3)/(-1*G$4))))</f>
+        <f t="shared" ref="G6:G13" si="0">G$1+G$2*(1/(1+EXP(($A6-G$3)/(-1*G$4))))</f>
         <v>104.61981689557548</v>
       </c>
       <c r="H6" s="2">
@@ -7221,7 +7383,7 @@
         <v>104.6</v>
       </c>
       <c r="G7" s="4">
-        <f>G$1+G$2*(1/(1+EXP(($A7-G$3)/(-1*G$4))))</f>
+        <f t="shared" si="0"/>
         <v>102.99154357040497</v>
       </c>
       <c r="H7" s="2">
@@ -7249,7 +7411,7 @@
         <v>100.23</v>
       </c>
       <c r="G8" s="4">
-        <f>G$1+G$2*(1/(1+EXP(($A8-G$3)/(-1*G$4))))</f>
+        <f t="shared" si="0"/>
         <v>96.307265875531698</v>
       </c>
       <c r="H8" s="2">
@@ -7277,7 +7439,7 @@
         <v>72.38</v>
       </c>
       <c r="G9" s="4">
-        <f>G$1+G$2*(1/(1+EXP(($A9-G$3)/(-1*G$4))))</f>
+        <f t="shared" si="0"/>
         <v>74.704517883544511</v>
       </c>
       <c r="H9" s="2">
@@ -7305,7 +7467,7 @@
         <v>20.5</v>
       </c>
       <c r="G10" s="4">
-        <f>G$1+G$2*(1/(1+EXP(($A10-G$3)/(-1*G$4))))</f>
+        <f t="shared" si="0"/>
         <v>37.43395317425162</v>
       </c>
       <c r="H10" s="2">
@@ -7333,7 +7495,7 @@
         <v>2.92</v>
       </c>
       <c r="G11" s="4">
-        <f>G$1+G$2*(1/(1+EXP(($A11-G$3)/(-1*G$4))))</f>
+        <f t="shared" si="0"/>
         <v>11.781020001246118</v>
       </c>
       <c r="H11" s="2">
@@ -7361,7 +7523,7 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="G12" s="4">
-        <f>G$1+G$2*(1/(1+EXP(($A12-G$3)/(-1*G$4))))</f>
+        <f t="shared" si="0"/>
         <v>3.112972801378449</v>
       </c>
       <c r="H12" s="2">
@@ -7389,7 +7551,7 @@
         <v>0.3</v>
       </c>
       <c r="G13" s="4">
-        <f>G$1+G$2*(1/(1+EXP(($A13-G$3)/(-1*G$4))))</f>
+        <f t="shared" si="0"/>
         <v>0.94404294011634238</v>
       </c>
       <c r="H13" s="2">
@@ -7398,7 +7560,116 @@
       <c r="I13" s="5"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C14" s="2"/>
       <c r="I14" s="5"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>0</v>
+      </c>
+      <c r="B15" s="3">
+        <v>105.1</v>
+      </c>
+      <c r="C15" s="2">
+        <f>C$1+C$2*(1/(1+EXP(($A15-C$3)/(-1*C$4))))</f>
+        <v>103.73943847719816</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2">
+        <f t="shared" ref="D15:E20" si="1">E$1+E$2*(1/(1+EXP(($A15-E$3)/(-1*E$4))))</f>
+        <v>105.03903826541399</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>9.9994070902634192E-6</v>
+      </c>
+      <c r="B16" s="2">
+        <f>B15-(2.8*A16)</f>
+        <v>105.09997200166015</v>
+      </c>
+      <c r="C16" s="2">
+        <f>C$1+C$2*(1/(1+EXP(($A16-C$3)/(-1*C$4))))</f>
+        <v>103.73940820331256</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2">
+        <f t="shared" si="1"/>
+        <v>105.03903556022327</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>0.5</v>
+      </c>
+      <c r="B17" s="3">
+        <f>B7</f>
+        <v>103.7</v>
+      </c>
+      <c r="C17" s="2">
+        <f>C$1+C$2*(1/(1+EXP(($A17-C$3)/(-1*C$4))))</f>
+        <v>101.01058733442666</v>
+      </c>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2">
+        <f t="shared" si="1"/>
+        <v>104.54129705775162</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>1</v>
+      </c>
+      <c r="B18" s="3">
+        <f>B8</f>
+        <v>98.4</v>
+      </c>
+      <c r="C18" s="2">
+        <f t="shared" ref="C18:C20" si="2">C$1+C$2*(1/(1+EXP(($A18-C$3)/(-1*C$4))))</f>
+        <v>93.426218607705962</v>
+      </c>
+      <c r="E18" s="2">
+        <f t="shared" si="1"/>
+        <v>100.17084695591934</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>1.23</v>
+      </c>
+      <c r="B19" s="3">
+        <f>124.2-(25.8*A19)</f>
+        <v>92.466000000000008</v>
+      </c>
+      <c r="C19" s="2">
+        <f t="shared" si="2"/>
+        <v>86.87294455025453</v>
+      </c>
+      <c r="E19" s="2">
+        <f t="shared" si="1"/>
+        <v>92.468764101859207</v>
+      </c>
+      <c r="F19" s="13">
+        <f>B19-E19</f>
+        <v>-2.7641018591992861E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>1.5</v>
+      </c>
+      <c r="B20" s="3">
+        <f>B9</f>
+        <v>85.5</v>
+      </c>
+      <c r="C20" s="2">
+        <f t="shared" si="2"/>
+        <v>75.859614230350189</v>
+      </c>
+      <c r="E20" s="2">
+        <f t="shared" si="1"/>
+        <v>72.35266118185983</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7441,25 +7712,25 @@
       <c r="B3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="8">
         <v>12.269617706237399</v>
       </c>
-      <c r="D3" s="7"/>
+      <c r="D3" s="8"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="8">
         <v>1.8809533698123699</v>
       </c>
-      <c r="D4" s="7"/>
+      <c r="D4" s="8"/>
     </row>
     <row r="5" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="8"/>
+      <c r="B5" s="9"/>
       <c r="C5" s="2">
         <v>2.7</v>
       </c>
@@ -7469,16 +7740,16 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="7" t="s">
         <v>17</v>
       </c>
     </row>
@@ -7658,25 +7929,25 @@
       <c r="B3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="8">
         <v>1.9211045364891499</v>
       </c>
-      <c r="D3" s="7"/>
+      <c r="D3" s="8"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="8">
         <v>-0.443561566638489</v>
       </c>
-      <c r="D4" s="7"/>
+      <c r="D4" s="8"/>
     </row>
     <row r="5" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="8"/>
+      <c r="B5" s="9"/>
       <c r="C5" s="2">
         <v>-0.33</v>
       </c>
@@ -7686,16 +7957,16 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="7" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>